<commit_message>
feat: add packet 0x69 (move_blocked) and bulletin/mail_box updates
- Add request::move_blocked (0x69) protocol and no-op handler; register in server and protocol.h
- Update bulletin message protocol, mail_box, listener, and enum.bulletin.xlsx
- Adjust bulletin handler and bulletin_message serialization; sync Model.cs
</commit_message>
<xml_diff>
--- a/resources/table/enum.bulletin.xlsx
+++ b/resources/table/enum.bulletin.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B2014F-BA83-4451-8E63-793E69F95D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{164E6A09-4A77-497A-9C9F-753A6ED9A10E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{E3DF90E4-1439-4BA6-8481-C5727015A5CB}"/>
   </bookViews>
   <sheets>
     <sheet name="BULLETIN_ACTION" sheetId="1" r:id="rId1"/>
     <sheet name="BULLETIN_BUTTON_ENABLE" sheetId="2" r:id="rId2"/>
     <sheet name="MAIL_BUTTON_ENABLE" sheetId="3" r:id="rId3"/>
+    <sheet name="BULLETIN_MESSAGE_TYPE" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="28">
   <si>
     <t>0x01</t>
   </si>
@@ -108,6 +109,22 @@
   </si>
   <si>
     <t>0x01</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WRITE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>READ</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DELETE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x07</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -676,4 +693,42 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33E74426-ED2E-4524-AAE1-1BD5DED1CE44}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>